<commit_message>
Lead finder: per-customer CRM, appointment calendar, recommendation reasons, main logo
- Each customer: sales stage, contact person, need-appointment flag, next step, notes
- Activity log (call/LINE/email/visit/note) with who we talked to, outcome and who logged it
- Appointment calendar (month view + agenda), .ics export to the phone calendar
- Why-recommended reasons per hotel (page + xlsx) and an overview of the selection
- Main keys logo; text autosaves while typing and open customer/drafts survive pull-to-refresh

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NpbPmSXoFQBETjhnTs3cz6
</commit_message>
<xml_diff>
--- a/hotel-leads/bangkok-cloudbeds-hotels.xlsx
+++ b/hotel-leads/bangkok-cloudbeds-hotels.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="แบ่งตามราคา" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'รายชื่อทั้งหมด'!$A$1:$R$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'รายชื่อทั้งหมด'!$A$1:$S$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'สรุปตามเขต'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'แบ่งตามดาว'!$A$1:$J$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'แบ่งตามรีวิว'!$A$1:$J$53</definedName>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R53"/>
+  <dimension ref="A1:S53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -460,7 +460,8 @@
     <col width="9" customWidth="1" min="15" max="15"/>
     <col width="45" customWidth="1" min="16" max="16"/>
     <col width="48" customWidth="1" min="17" max="17"/>
-    <col width="45" customWidth="1" min="18" max="18"/>
+    <col width="70" customWidth="1" min="18" max="18"/>
+    <col width="45" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -551,6 +552,11 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>เหตุผลที่เสนอ</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>หมายเหตุ</t>
         </is>
       </c>
@@ -623,6 +629,11 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดใหญ่ 120 ห้อง งานหน้าบ้านและการจองเยอะ / ระดับ 4 ดาว มีงบลงทุนระบบ / ราคา ~1,400 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (คลองเตย) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
           <t>ชื่อเดิม Aspira Grand Regency · ตึกเก่า · ดาวประกาศเอง</t>
         </is>
       </c>
@@ -699,6 +710,11 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดเล็ก 10 ห้อง คุยกับเจ้าของได้ตรง ตัดสินใจเร็ว / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
           <t>เปิดปี 2022 · ใกล้ BTS หมอชิต</t>
         </is>
       </c>
@@ -767,6 +783,11 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / คะแนนรีวิว 9.0 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ใกล้สนามบินดอนเมือง แขกเข้าออกเร็ว ต้องจัดการห้องไว / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
           <t>~1.1 กม. จากสนามบิน DMK</t>
         </is>
       </c>
@@ -831,6 +852,11 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดใหญ่ 60 ห้อง งานหน้าบ้านและการจองเยอะ / ใกล้สนามบินดอนเมือง แขกเข้าออกเร็ว ต้องจัดการห้องไว / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
           <t>ใกล้สนามบินดอนเมือง · มีร้านอาหาร</t>
         </is>
       </c>
@@ -903,6 +929,11 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / มีหลายสาขาหรือมีโรงแรมพี่น้อง คุยครั้งเดียวมีโอกาสได้หลายแห่ง / ขนาดใหญ่ 388 ห้อง งานหน้าบ้านและการจองเยอะ / คะแนนรีวิว 9.0 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~1,600 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
           <t>เครือ StayBangkok · ใกล้ MRT · ไม่รวมอาหารเช้า</t>
         </is>
       </c>
@@ -970,6 +1001,11 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดกลาง 29 ห้อง กำลังโต / ราคา ~1,250 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
           <t>เดิน ~10 นาที MRT ห้วยขวาง</t>
         </is>
       </c>
@@ -1047,6 +1083,11 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดเล็ก 19 ห้อง คุยกับเจ้าของได้ตรง ตัดสินใจเร็ว / คะแนนรีวิว 9.5 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~1,800 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
           <t>adults only · ใกล้ท่าเรือเทเวศร์</t>
         </is>
       </c>
@@ -1116,6 +1157,11 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดเล็ก 3 ห้อง คุยกับเจ้าของได้ตรง ตัดสินใจเร็ว / คะแนนรีวิว 9.7 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~3,900 ฿/คืน กลุ่มพรีเมียม รายได้ต่อห้องสูง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
           <t>ติด MRT อิสรภาพ · มีสระ · ห้องน้อยมาก</t>
         </is>
       </c>
@@ -1183,6 +1229,11 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดเล็ก 5 ห้อง คุยกับเจ้าของได้ตรง ตัดสินใจเร็ว / คะแนนรีวิว 10.0 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~2,500 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (บางรัก) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
           <t>loft · pet-friendly</t>
         </is>
       </c>
@@ -1246,6 +1297,11 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / คะแนนรีวิว 9.0 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~1,120 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (บางรัก) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
           <t>มีทั้งเตียงรวมและห้องส่วนตัว</t>
         </is>
       </c>
@@ -1312,6 +1368,11 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 1,785 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / อยู่ย่านท่องเที่ยวหลัก (บางรัก) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
           <t>มีสระว่ายน้ำดาดฟ้า</t>
         </is>
       </c>
@@ -1376,6 +1437,11 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดกลาง 30 ห้อง กำลังโต / รีวิว 2,281 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~1,780 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (บางรัก) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
           <t>รีโนเวทปี 2024 · สระดาดฟ้า</t>
         </is>
       </c>
@@ -1440,6 +1506,11 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดใหญ่ 72 ห้อง งานหน้าบ้านและการจองเยอะ / รีวิว 2,197 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~890 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (บางรัก) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
           <t>มีสระว่ายน้ำ · ไม่มีอาหารเช้า</t>
         </is>
       </c>
@@ -1509,6 +1580,11 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดเล็ก 17 ห้อง คุยกับเจ้าของได้ตรง ตัดสินใจเร็ว / รีวิว 1,420 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / อยู่ย่านท่องเที่ยวหลัก (บางรัก) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
           <t>รีวิว Hostelworld ต่ำมาก (2.6)</t>
         </is>
       </c>
@@ -1570,6 +1646,11 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 2,442 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / คะแนนรีวิว 9.4 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~880 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (ปทุมวัน) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
           <t>design hostel ใกล้ MRT หัวลำโพง</t>
         </is>
       </c>
@@ -1638,6 +1719,11 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / คะแนนรีวิว 9.3 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / อยู่ย่านท่องเที่ยวหลัก (ปทุมวัน) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
           <t>ใกล้หัวลำโพง</t>
         </is>
       </c>
@@ -1709,6 +1795,11 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 3,890 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~1,550 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (ปทุมวัน) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
           <t>ใกล้ BTS สนามกีฬาฯ/สยาม</t>
         </is>
       </c>
@@ -1778,6 +1869,11 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดเล็ก 9 ห้อง คุยกับเจ้าของได้ตรง ตัดสินใจเร็ว / ราคา ~1,500 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (ปทุมวัน) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
           <t>ตรงข้ามสวนลุมฯ</t>
         </is>
       </c>
@@ -1849,6 +1945,11 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ราคา ~1,150 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (ปทุมวัน) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
           <t>~1 กม. MBK</t>
         </is>
       </c>
@@ -1918,6 +2019,11 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / มีหลายสาขาหรือมีโรงแรมพี่น้อง คุยครั้งเดียวมีโอกาสได้หลายแห่ง / ขนาดกลาง 24 ห้อง กำลังโต / คะแนนรีวิว 9.8 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~1,800 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
           <t>ใกล้อนุสาวรีย์ประชาธิปไตย · เครือเดียวกับ Siri Grand</t>
         </is>
       </c>
@@ -1989,6 +2095,11 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 2,778 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / คะแนนรีวิว 9.7 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
           <t>rooftop bar</t>
         </is>
       </c>
@@ -2060,6 +2171,11 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 9,600 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / คะแนนรีวิว 9.3 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
           <t>หอพักใหญ่ 22 เตียง</t>
         </is>
       </c>
@@ -2126,6 +2242,11 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / คะแนนรีวิว 9.2 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~2,400 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
           <t>มีสระ · เจ้าของเดียวกับ Siri Ratchadamnoen</t>
         </is>
       </c>
@@ -2184,6 +2305,11 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 1,592 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / คะแนนรีวิว 9.2 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
           <t>party hostel 18-35</t>
         </is>
       </c>
@@ -2247,6 +2373,11 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / คะแนนรีวิว 9.1 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~1,100 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
           <t>แคปซูล · rooftop bar</t>
         </is>
       </c>
@@ -2318,6 +2449,11 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ระดับ 4 ดาว มีงบลงทุนระบบ / ราคา ~2,000 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
           <t>ชื่อเดิม The Ember · ลิงก์จาก 2023 ควรเช็กว่ายังใช้</t>
         </is>
       </c>
@@ -2384,6 +2520,11 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 1,140 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
           <t>adults only · แคปซูล</t>
         </is>
       </c>
@@ -2453,6 +2594,11 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ราคา ~1,200 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
           <t>มีสระ+ฟิตเนส</t>
         </is>
       </c>
@@ -2519,6 +2665,11 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ราคา ~1,100 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
           <t>ใกล้เสาชิงช้า</t>
         </is>
       </c>
@@ -2596,6 +2747,11 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดใหญ่ 55 ห้อง งานหน้าบ้านและการจองเยอะ / รีวิว 2,108 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~1,100 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
           <t>มีสระ+ร้านอาหาร</t>
         </is>
       </c>
@@ -2662,6 +2818,11 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ราคา ~900 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
           <t>ใกล้สะพานพระราม 8</t>
         </is>
       </c>
@@ -2728,6 +2889,11 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 2,852 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~880 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
           <t>มีสระ · บจก. HERE THE WORLD</t>
         </is>
       </c>
@@ -2804,6 +2970,11 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 7,235 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~1,250 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
           <t>มีห้องส่วนตัว+หอพัก</t>
         </is>
       </c>
@@ -2883,6 +3054,11 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 1,817 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / อยู่ย่านท่องเที่ยวหลัก (พระนคร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
           <t>adults only</t>
         </is>
       </c>
@@ -2938,6 +3114,11 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / อยู่ย่านท่องเที่ยวหลัก (ราชเทวี) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
           <t>รวมอาหารเช้า</t>
         </is>
       </c>
@@ -3003,6 +3184,11 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / อยู่ย่านท่องเที่ยวหลัก (ราชเทวี) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
           <t>เดิน 3 นาทีอนุสาวรีย์ชัยฯ</t>
         </is>
       </c>
@@ -3072,6 +3258,11 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ราคา ~1,500 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (ราชเทวี) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
           <t>ย่านอนุสาวรีย์ชัยฯ</t>
         </is>
       </c>
@@ -3139,6 +3330,11 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดใหญ่ 94 ห้อง งานหน้าบ้านและการจองเยอะ / รีวิว 1,926 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~910 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (ราชเทวี) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
           <t>ใกล้ประตูน้ำ/แพลทินัม</t>
         </is>
       </c>
@@ -3210,6 +3406,11 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / อยู่ย่านท่องเที่ยวหลัก (ราชเทวี) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
           <t>~570 ม. BTS อนุสาวรีย์ชัยฯ</t>
         </is>
       </c>
@@ -3287,6 +3488,11 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดกลาง 25 ห้อง กำลังโต / รีวิว 1,190 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / อยู่ย่านท่องเที่ยวหลัก (ราชเทวี) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
           <t>อาหารเช้า 150 บาท</t>
         </is>
       </c>
@@ -3356,6 +3562,11 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 1,082 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / คะแนนรีวิว 9.0 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / ราคา ~1,190 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (วัฒนา) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
           <t>ใกล้ Terminal 21</t>
         </is>
       </c>
@@ -3415,6 +3626,11 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดกลาง 21 ห้อง กำลังโต / อยู่ย่านท่องเที่ยวหลัก (วัฒนา) แข่งขันสูง ต้องการเครื่องมือช่วยขาย</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
           <t>ใช้ Cloudbeds โดเมน us2.cloudbeds.com</t>
         </is>
       </c>
@@ -3488,6 +3704,11 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 1,129 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / อยู่ย่านท่องเที่ยวหลัก (วัฒนา) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
           <t>ใกล้ BTS พร้อมพงษ์</t>
         </is>
       </c>
@@ -3552,6 +3773,11 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 1,548 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~1,020 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (วัฒนา) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
           <t>ชื่อเดิม Serene Asoke Suites</t>
         </is>
       </c>
@@ -3615,6 +3841,11 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 2,741 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / อยู่ย่านท่องเที่ยวหลัก (วัฒนา) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
           <t>เดิน 5 นาที BTS อโศก</t>
         </is>
       </c>
@@ -3679,6 +3910,11 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ราคา ~920 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (วัฒนา) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเบอร์โทร ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
           <t>เดิน 7 นาที BTS พร้อมพงษ์</t>
         </is>
       </c>
@@ -3753,6 +3989,11 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / คะแนนรีวิว 6.4 ค่อนข้างต่ำ มีจุดให้ช่วยปรับปรุงบริการ / ราคา ~920 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (วัฒนา) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีเว็บไซต์ของตัวเอง ให้ความสำคัญกับการจองตรง / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
           <t>ไม่มีลิฟต์ · 50 ม. BTS ทองหล่อ</t>
         </is>
       </c>
@@ -3806,6 +4047,11 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / อยู่ย่านท่องเที่ยวหลัก (วัฒนา) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
           <t>น่าจะเปิดใหม่ ยังไม่มีรีวิว</t>
         </is>
       </c>
@@ -3875,6 +4121,11 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / คะแนนรีวิว 9.3 ดีเยี่ยม ใส่ใจคุณภาพ พร้อมลงทุนต่อ / อยู่ย่านท่องเที่ยวหลัก (สัมพันธวงศ์) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
           <t>ใกล้ River City</t>
         </is>
       </c>
@@ -3941,6 +4192,11 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / รีวิว 1,774 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~880 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (สัมพันธวงศ์) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
           <t>เยาวราช · รับเงินสดเท่านั้น</t>
         </is>
       </c>
@@ -4012,6 +4268,11 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดกลาง 32 ห้อง กำลังโต / อยู่ย่านท่องเที่ยวหลัก (สาทร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
           <t>ตึกแถวเก่า 7 คูหา · ใกล้ BTS สะพานตากสิน</t>
         </is>
       </c>
@@ -4084,12 +4345,17 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
+          <t>ใช้ Cloudbeds อยู่แล้ว (เจอหน้าจองตรงบน Cloudbeds) เปิดรับระบบออนไลน์และจ่ายค่าซอฟต์แวร์อยู่ / ขนาดใหญ่ 156 ห้อง งานหน้าบ้านและการจองเยอะ / ระดับ 5 ดาว มีงบลงทุนระบบ / รีวิว 4,554 รายการ แขกเข้าพักต่อเนื่อง ธุรกิจมีรายได้สม่ำเสมอ / ราคา ~1,900 ฿/คืน กลุ่มราคากลาง ตรงกลุ่มเป้าหมาย / อยู่ย่านท่องเที่ยวหลัก (สาทร) แข่งขันสูง ต้องการเครื่องมือช่วยขาย / มีทั้งเบอร์โทรและอีเมล ติดต่อได้ทันที</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
           <t>ดาวประกาศเองบนหน้าจอง ยังไม่ยืนยัน · ห้องมีครัว</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R53"/>
+  <autoFilter ref="A1:S53"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>

</xml_diff>